<commit_message>
Read product names left of SP_SPCD and SP_SPCD1 in the relation sheet
The relation sheet now carries two name columns, each directly left of
its code (주보종명 | SP_SPCD | 개별상품명 | SP_SPCD1). stat_builder picks
them by position, so identical headers such as two '상품명' columns no
longer collapse into one, and shows them beside the codes in the review
sheet. Files without the name columns still run, with a note in the log.
The example template follows the new layout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHEdtSnidyfERzeafRkXoB
</commit_message>
<xml_diff>
--- a/web/sample/sample_revision.xlsx
+++ b/web/sample/sample_revision.xlsx
@@ -1055,113 +1055,144 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>주보종명</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>SP_SPCD</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>개별상품명</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>SP_SPCD1</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>상품명</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>(무)예제건강보험Ⅱ</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>A200</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>(무)예제암진단특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>A2001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>(무)예제암진단특약Ⅱ</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>(무)예제건강보험Ⅱ</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>A200</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>(무)예제상해보장특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>A2002</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>(무)예제상해보장특약Ⅱ</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>(무)예제건강보험Ⅱ</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>A200</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>(무)예제납입면제특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>A2003</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>(무)예제납입면제특약Ⅱ</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>(무)예제건강보험Ⅱ</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>A200</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>(무)예제수술특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>A2006</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>(무)예제수술특약Ⅱ</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>(무)예제건강보험Ⅱ</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>A200</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>(무)예제간병특약(신규)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>A2008</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>(무)예제간병특약(신규)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Put both product-name columns before SP_SPCD in the relation sheet
Layout is now 주보종명 | 개별상품명 | SP_SPCD | SP_SPCD1. stat_builder
reads the two columns directly left of SP_SPCD in that order, or the
columns headed 주보종명 / 개별상품명 wherever they are. Example template
and page text follow the new order.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHEdtSnidyfERzeafRkXoB
</commit_message>
<xml_diff>
--- a/web/sample/sample_revision.xlsx
+++ b/web/sample/sample_revision.xlsx
@@ -1072,12 +1072,12 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>개별상품명</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>SP_SPCD</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>개별상품명</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -1092,14 +1092,14 @@
           <t>(무)예제건강보험Ⅱ</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>(무)예제암진단특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>A200</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>(무)예제암진단특약Ⅱ</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1114,14 +1114,14 @@
           <t>(무)예제건강보험Ⅱ</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>(무)예제상해보장특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>A200</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>(무)예제상해보장특약Ⅱ</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1136,14 +1136,14 @@
           <t>(무)예제건강보험Ⅱ</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>(무)예제납입면제특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>A200</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>(무)예제납입면제특약Ⅱ</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1158,14 +1158,14 @@
           <t>(무)예제건강보험Ⅱ</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>(무)예제수술특약Ⅱ</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>A200</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>(무)예제수술특약Ⅱ</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1180,14 +1180,14 @@
           <t>(무)예제건강보험Ⅱ</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>(무)예제간병특약(신규)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>A200</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>(무)예제간병특약(신규)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Replace 납입주기 with 지급주기 (100 / 211) in the draft table
The draft column was the premium payment cycle; the statistics table
needs the benefit payment cycle (PAY_TERM1). get_pay_term() returns 211
when the reason/amount describes a fixed number of monthly payments
(매월 … n회, n회 월지급, n개월간 매월) and 100 otherwise. The column sits
after 지급율 like PAY_RATE1/PAY_TERM1; 납입주기 stays in 급부원문 for
reference and the matched wording goes to 근거_지급주기. Examples and
the info tab follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHEdtSnidyfERzeafRkXoB
</commit_message>
<xml_diff>
--- a/web/sample/sample_revision.xlsx
+++ b/web/sample/sample_revision.xlsx
@@ -708,8 +708,10 @@
       <c r="E3" t="n">
         <v>0.5</v>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G3" t="n">
         <v>1</v>
@@ -748,8 +750,10 @@
       <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="n">
-        <v>0</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -788,8 +792,10 @@
       <c r="E5" t="n">
         <v>0.2</v>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -828,8 +834,10 @@
       <c r="E6" t="n">
         <v>0.02</v>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -868,8 +876,10 @@
       <c r="E7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" t="n">
-        <v>0</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -908,8 +918,10 @@
       <c r="E8" t="n">
         <v>0.1</v>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -948,8 +960,10 @@
       <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" t="n">
-        <v>0</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G9" t="n">
         <v>1</v>
@@ -988,8 +1002,10 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="n">
-        <v>0</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="G10" t="n">
         <v>1</v>
@@ -1028,8 +1044,10 @@
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="n">
-        <v>0</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
       </c>
       <c r="G11" t="n">
         <v>1</v>

</xml_diff>